<commit_message>
update to isoorbi 1.5.1
</commit_message>
<xml_diff>
--- a/output/table2_nitrate_ratios.xlsx
+++ b/output/table2_nitrate_ratios.xlsx
@@ -1,61 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25427"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kantn\Dropbox\Dokumenty\US_Boulder\GitHub\2023_kantnerova_et_al\output\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073BA02D-E850-437E-8E7A-BA3C03031F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="10980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="dataset" sheetId="1" r:id="rId1"/>
+    <sheet name="dataset" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
-  <si>
-    <t>sample_name</t>
-  </si>
-  <si>
-    <t>isotopocule_ratio</t>
-  </si>
-  <si>
-    <t>ratio_expected</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>ratio_raw_mean</t>
-  </si>
-  <si>
-    <t>ratio_raw_sdev_rel</t>
-  </si>
-  <si>
-    <t>ratio_corrected_mean</t>
-  </si>
-  <si>
-    <t>ratio_corrected_sdev_rel</t>
-  </si>
-  <si>
-    <t>USGS32</t>
-  </si>
-  <si>
-    <t>15N/M0</t>
-  </si>
-  <si>
-    <t>17O/M0</t>
-  </si>
-  <si>
-    <t>18O/M0</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t xml:space="preserve">sample_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">isotopocule_ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratio_expected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratio_raw_mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratio_raw_sdev_rel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratio_corrected_mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratio_corrected_sdev_rel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USGS32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15N/M0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17O/M0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18O/M0</t>
   </si>
 </sst>
 </file>
@@ -63,10 +55,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0000000"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -75,22 +67,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <b/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -110,32 +95,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -417,21 +389,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="4" width="1.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="8" width="24.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="17.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="1.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="24.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,85 +429,85 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4">
-        <v>4.33768E-3</v>
-      </c>
-      <c r="D2" s="2">
+      <c r="C2" s="3" t="n">
+        <v>0.00433768</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E2" s="4">
-        <v>5.1775316666666698E-3</v>
-      </c>
-      <c r="F2" s="5">
-        <v>1.0957164154855501E-3</v>
-      </c>
-      <c r="G2" s="4">
-        <v>4.3452877054515598E-3</v>
-      </c>
-      <c r="H2" s="5">
-        <v>1.03917980691397E-3</v>
+      <c r="E2" s="3" t="n">
+        <v>0.00517753166666667</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.00109571641548555</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.00434528770545156</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.00103917980691397</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="4">
-        <v>1.1550480000000001E-3</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="C3" s="3" t="n">
+        <v>0.001155048</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="4">
-        <v>1.38093166666667E-3</v>
-      </c>
-      <c r="F3" s="5">
-        <v>2.4076108802834799E-3</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1.1538485507992099E-3</v>
-      </c>
-      <c r="H3" s="5">
-        <v>2.3259063394795798E-3</v>
+      <c r="E3" s="3" t="n">
+        <v>0.00138093166666667</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.00240761088028348</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.00115384855079921</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.00232590633947958</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4">
-        <v>6.1706112000000004E-3</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="C4" s="3" t="n">
+        <v>0.0061706112</v>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E4" s="4">
-        <v>8.8537716666666696E-3</v>
-      </c>
-      <c r="F4" s="5">
-        <v>1.6771778093587399E-3</v>
-      </c>
-      <c r="G4" s="4">
-        <v>6.1798331159733499E-3</v>
-      </c>
-      <c r="H4" s="5">
-        <v>1.41070780905578E-3</v>
+      <c r="E4" s="3" t="n">
+        <v>0.00885377166666667</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.00167717780935874</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.00617983311597335</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.00141070780905578</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="C5" s="3"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
@@ -545,6 +517,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>